<commit_message>
update profile list and change link to github issue e0574496f4f02093519f9138e8b517ef7113e571
</commit_message>
<xml_diff>
--- a/ig/nr-deploy-1.0.0-ballot/CodeSystem-type-systeme-information-cs.xlsx
+++ b/ig/nr-deploy-1.0.0-ballot/CodeSystem-type-systeme-information-cs.xlsx
@@ -24,7 +24,7 @@
     <t>URL</t>
   </si>
   <si>
-    <t>http://interop.esante.gouv.fr/ig/fhir/annuaire/CodeSystem/type-systeme-information-cs</t>
+    <t>https://interop.esante.gouv.fr/ig/fhir/annuaire/CodeSystem/type-systeme-information-cs</t>
   </si>
   <si>
     <t>Version</t>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2023-06-02T12:29:31+00:00</t>
+    <t>2023-06-02T14:39:58+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>